<commit_message>
docs(handover): Sentinel gap matrix statuses -> WORKING/PARTIAL/MISSING/BLOCKED vocabulary
Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/afruheritage-platform/uat-package/SENTINEL_CUSTOMER_ADMIN_GAP_MATRIX.xlsx
+++ b/afruheritage-platform/uat-package/SENTINEL_CUSTOMER_ADMIN_GAP_MATRIX.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>FIXED + VERIFIED</t>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>GAP (backend missing)</t>
+          <t>MISSING</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>GAP (backend missing)</t>
+          <t>MISSING</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>GAP (unmounted)</t>
+          <t>MISSING</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1437,49 +1437,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Remaining gaps</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Payment refund/dispute</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>No CP backend for refund/dispute — calls return honest 404</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Runner restart/shutdown/metrics</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>No CP backend — previously fake-succeeded on mock data</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Tenant detail stats</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Router not mounted; placeholder zeros</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(handover): action-level Sentinel verification — flag/ticket/KYC writes confirmed, tenant-flags + audit gaps logged
Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/afruheritage-platform/uat-package/SENTINEL_CUSTOMER_ADMIN_GAP_MATRIX.xlsx
+++ b/afruheritage-platform/uat-package/SENTINEL_CUSTOMER_ADMIN_GAP_MATRIX.xlsx
@@ -34,7 +34,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +54,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -95,6 +100,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -463,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1245,27 +1253,27 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Stale bundle</t>
+          <t>Tickets — status update</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Navigation missing Payments/Shipments/Fleetbase/FeatureFlags/Diagnostics</t>
+          <t>Admin ticket status transitions persist</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>deployed static bundle</t>
+          <t>PATCH /sentinel/tickets/{id}/status?status=</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Deployed bundle predated source routes</t>
+          <t>Write path untested during page recon</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Rebuilt Next static export, redeployed</t>
+          <t>Verified live: open→resolved→open persisted; invalid status→400; unknown id→404</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1277,94 +1285,286 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Payment refund/dispute</t>
+          <t>KYC — approve action</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Refund and dispute actions</t>
+          <t>Admin KYC decision persists to DB</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>POST /sentinel/payments/{id}/refund|dispute</t>
+          <t>POST /sentinel/kyc/approve/{id}</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>No CP backend for refund/dispute — calls return honest 404</t>
+          <t>Write path untested during page recon</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Deferred — needs CP refund/dispute endpoints</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Verified on cert-test record: pending→approved in DB</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Runner restart/shutdown/metrics</t>
+          <t>Feature Flags — global write</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Runner lifecycle controls</t>
+          <t>Global per-key toggle persists</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>POST /sentinel/runners/{id}/restart|shutdown</t>
+          <t>PATCH /sentinel/feature-flags/global/{key}</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>No CP backend — previously fake-succeeded on mock data</t>
+          <t>Write path untested during page recon</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Now returns honest 501 until CP supports it</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>csv_import toggled off→verified persisted→restored on</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>WORKING</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Feature Flags — tenant scope</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Per-tenant flag view/manage</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>GET/PATCH /sentinel/feature-flags/tenant/{id}</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Control plane returns 'Not Found' — no tenant-flag backend</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Needs CP tenant-flag endpoints (global flags only today)</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Audit coverage</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Admin action audit trail</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>admin_audit_logs table</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Only admin.login + runners.listed audited; CP-proxied mutations (KYC approve, flag toggle, ticket status, tenant actions) write no audit row</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Needs audit middleware/decorator on all sentinel write routes</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Flag-state consistency</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Global flags vs deferred features</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>marketplace_enabled, vendor_registration = enabled</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Deferred features' global flags are enabled — inert today (no customer nav) but inconsistent with Coming Soon register</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Review flag defaults or document that flags are inert</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Stale bundle</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Navigation missing Payments/Shipments/Fleetbase/FeatureFlags/Diagnostics</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>deployed static bundle</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Deployed bundle predated source routes</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Rebuilt Next static export, redeployed</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>WORKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Payment refund/dispute</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Refund and dispute actions</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>POST /sentinel/payments/{id}/refund|dispute</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>No CP backend for refund/dispute — calls return honest 404</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Deferred — needs CP refund/dispute endpoints</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Runner restart/shutdown/metrics</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Runner lifecycle controls</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>POST /sentinel/runners/{id}/restart|shutdown</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>No CP backend — previously fake-succeeded on mock data</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Now returns honest 501 until CP supports it</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>Tenant detail stats</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Per-tenant shipments/storage/API metrics</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>tenants_advanced.py</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Router not mounted; placeholder zeros</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Unmounted dead code — needs real implementation if enabled</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1389,7 +1589,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
@@ -1407,7 +1607,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -1417,7 +1617,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -1441,7 +1641,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Remaining gaps</t>
         </is>

</xml_diff>